<commit_message>
feat(blog): add video support to blog posts with migration and DTO updates
This commit introduces a new migration to add a 'videos' column to the 'blog_posts' table, replacing the 'featured_video' column. It updates the blog post DTOs to include support for multiple video types (file and URL) and modifies the blog import script to initialize the 'videos' field. Additionally, it enhances the blog post entity and service to handle video uploads and normalization, improving the overall media management for blog posts.
</commit_message>
<xml_diff>
--- a/docs/Master-Data-Sheets/cureka_category_page_descriptions_above the fold.xlsx
+++ b/docs/Master-Data-Sheets/cureka_category_page_descriptions_above the fold.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" firstSheet="1" activeTab="6"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11760" firstSheet="1" activeTab="6"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="healthcare devices" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Herbal &amp; Ayurvedha" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="vitamins &amp; nutrition" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="personal care" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="baby care" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="sexual wellness" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="women care" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Sheet1" state="visible" r:id="rId11"/>
+    <sheet name="healthcare devices" sheetId="1" r:id="rId1"/>
+    <sheet name="Herbal &amp; Ayurvedha" sheetId="2" r:id="rId2"/>
+    <sheet name="vitamins &amp; nutrition" sheetId="3" r:id="rId3"/>
+    <sheet name="personal care" sheetId="4" r:id="rId4"/>
+    <sheet name="baby care" sheetId="5" r:id="rId5"/>
+    <sheet name="sexual wellness" sheetId="6" r:id="rId6"/>
+    <sheet name="women care" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">'women care'!$A$1:$G$21</definedName>
@@ -4490,14 +4490,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -4522,10 +4522,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -4843,13 +4851,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4872,7 +4880,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -4895,7 +4903,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -4918,7 +4926,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -4941,7 +4949,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -4964,7 +4972,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="60" customHeight="1">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -4987,7 +4995,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -5010,7 +5018,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="60" customHeight="1">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -5033,7 +5041,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="60" customHeight="1">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -5056,7 +5064,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -5079,7 +5087,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -5102,7 +5110,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -5125,7 +5133,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1">
       <c r="A13" t="s">
         <v>76</v>
       </c>
@@ -5148,7 +5156,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1">
       <c r="A14" t="s">
         <v>82</v>
       </c>
@@ -5171,7 +5179,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1">
       <c r="A15" t="s">
         <v>88</v>
       </c>
@@ -5194,7 +5202,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1">
       <c r="A16" t="s">
         <v>95</v>
       </c>
@@ -5217,7 +5225,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1">
       <c r="A17" t="s">
         <v>101</v>
       </c>
@@ -5240,7 +5248,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -5263,7 +5271,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1">
       <c r="A19" t="s">
         <v>114</v>
       </c>
@@ -5286,7 +5294,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1">
       <c r="A20" t="s">
         <v>121</v>
       </c>
@@ -5309,7 +5317,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1">
       <c r="A21" t="s">
         <v>127</v>
       </c>
@@ -5332,7 +5340,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60" customHeight="1">
       <c r="A22" t="s">
         <v>134</v>
       </c>
@@ -5355,7 +5363,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" customHeight="1">
       <c r="A23" t="s">
         <v>141</v>
       </c>
@@ -5378,7 +5386,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" customHeight="1">
       <c r="A24" t="s">
         <v>147</v>
       </c>
@@ -5401,7 +5409,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" customHeight="1">
       <c r="A25" t="s">
         <v>154</v>
       </c>
@@ -5424,7 +5432,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" customHeight="1">
       <c r="A26" t="s">
         <v>161</v>
       </c>
@@ -5447,7 +5455,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" customHeight="1">
       <c r="A27" t="s">
         <v>167</v>
       </c>
@@ -5470,7 +5478,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="60" customHeight="1">
       <c r="A28" t="s">
         <v>173</v>
       </c>
@@ -5493,7 +5501,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="60" customHeight="1">
       <c r="A29" t="s">
         <v>176</v>
       </c>
@@ -5516,7 +5524,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="60" customHeight="1">
       <c r="A30" t="s">
         <v>182</v>
       </c>
@@ -5539,7 +5547,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60" customHeight="1">
       <c r="A31" t="s">
         <v>185</v>
       </c>
@@ -5562,7 +5570,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="32" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60" customHeight="1">
       <c r="A32" t="s">
         <v>193</v>
       </c>
@@ -5585,7 +5593,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="60" customHeight="1">
       <c r="A33" t="s">
         <v>199</v>
       </c>
@@ -5608,7 +5616,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="60" customHeight="1">
       <c r="A34" t="s">
         <v>205</v>
       </c>
@@ -5631,7 +5639,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="35" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="60" customHeight="1">
       <c r="A35" t="s">
         <v>212</v>
       </c>
@@ -5654,7 +5662,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="60" customHeight="1">
       <c r="A36" t="s">
         <v>219</v>
       </c>
@@ -5677,7 +5685,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="60" customHeight="1">
       <c r="A37" t="s">
         <v>225</v>
       </c>
@@ -5700,7 +5708,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="38" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="60" customHeight="1">
       <c r="A38" t="s">
         <v>232</v>
       </c>
@@ -5723,7 +5731,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="39" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="60" customHeight="1">
       <c r="A39" t="s">
         <v>238</v>
       </c>
@@ -5746,7 +5754,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="60" customHeight="1">
       <c r="A40" t="s">
         <v>245</v>
       </c>
@@ -5769,7 +5777,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="41" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="60" customHeight="1">
       <c r="A41" t="s">
         <v>252</v>
       </c>
@@ -5792,7 +5800,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="42" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="60" customHeight="1">
       <c r="A42" t="s">
         <v>259</v>
       </c>
@@ -5815,7 +5823,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="43" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="60" customHeight="1">
       <c r="A43" t="s">
         <v>266</v>
       </c>
@@ -5838,7 +5846,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="44" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="60" customHeight="1">
       <c r="A44" t="s">
         <v>272</v>
       </c>
@@ -5861,7 +5869,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="45" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="60" customHeight="1">
       <c r="A45" t="s">
         <v>278</v>
       </c>
@@ -5884,7 +5892,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="60" customHeight="1">
       <c r="A46" t="s">
         <v>284</v>
       </c>
@@ -5907,7 +5915,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="47" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="60" customHeight="1">
       <c r="A47" t="s">
         <v>290</v>
       </c>
@@ -5930,7 +5938,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="48" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="60" customHeight="1">
       <c r="A48" t="s">
         <v>296</v>
       </c>
@@ -5953,7 +5961,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="49" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="60" customHeight="1">
       <c r="A49" t="s">
         <v>302</v>
       </c>
@@ -5976,7 +5984,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="50" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="60" customHeight="1">
       <c r="A50" t="s">
         <v>309</v>
       </c>
@@ -5999,7 +6007,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="51" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="60" customHeight="1">
       <c r="A51" t="s">
         <v>316</v>
       </c>
@@ -6022,7 +6030,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="52" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="60" customHeight="1">
       <c r="A52" t="s">
         <v>322</v>
       </c>
@@ -6045,7 +6053,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="53" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="60" customHeight="1">
       <c r="A53" t="s">
         <v>329</v>
       </c>
@@ -6068,7 +6076,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="54" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="60" customHeight="1">
       <c r="A54" t="s">
         <v>335</v>
       </c>
@@ -6091,7 +6099,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="55" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="60" customHeight="1">
       <c r="A55" t="s">
         <v>341</v>
       </c>
@@ -6114,7 +6122,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="56" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="60" customHeight="1">
       <c r="A56" t="s">
         <v>347</v>
       </c>
@@ -6146,16 +6154,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="76" customWidth="1"/>
+    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="4" max="4" width="23.109375" customWidth="1"/>
     <col min="5" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -6178,7 +6187,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1">
       <c r="A2" t="s">
         <v>359</v>
       </c>
@@ -6201,7 +6210,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>366</v>
       </c>
@@ -6224,7 +6233,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>373</v>
       </c>
@@ -6247,7 +6256,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>380</v>
       </c>
@@ -6270,7 +6279,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="6" ht="64.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="64.5" customHeight="1">
       <c r="A6" t="s">
         <v>387</v>
       </c>
@@ -6293,7 +6302,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" t="s">
         <v>394</v>
       </c>
@@ -6316,7 +6325,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="60" customHeight="1">
       <c r="A8" t="s">
         <v>399</v>
       </c>
@@ -6339,7 +6348,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="60" customHeight="1">
       <c r="A9" t="s">
         <v>405</v>
       </c>
@@ -6362,7 +6371,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1">
       <c r="A10" t="s">
         <v>412</v>
       </c>
@@ -6385,7 +6394,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1">
       <c r="A11" t="s">
         <v>419</v>
       </c>
@@ -6408,7 +6417,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1">
       <c r="A12" t="s">
         <v>426</v>
       </c>
@@ -6431,7 +6440,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1">
       <c r="A13" t="s">
         <v>433</v>
       </c>
@@ -6454,7 +6463,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1">
       <c r="A14" t="s">
         <v>440</v>
       </c>
@@ -6477,7 +6486,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1">
       <c r="A15" t="s">
         <v>447</v>
       </c>
@@ -6500,7 +6509,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1">
       <c r="A16" t="s">
         <v>454</v>
       </c>
@@ -6523,7 +6532,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1">
       <c r="A17" t="s">
         <v>461</v>
       </c>
@@ -6546,7 +6555,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1">
       <c r="A18" t="s">
         <v>468</v>
       </c>
@@ -6569,7 +6578,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1">
       <c r="A19" t="s">
         <v>475</v>
       </c>
@@ -6592,7 +6601,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1">
       <c r="A20" t="s">
         <v>482</v>
       </c>
@@ -6615,7 +6624,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1">
       <c r="A21" t="s">
         <v>489</v>
       </c>
@@ -6641,22 +6650,22 @@
   </sheetData>
   <autoFilter ref="A1:G21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="0"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G41"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
     <col min="4" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -6679,7 +6688,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1">
       <c r="A2" t="s">
         <v>496</v>
       </c>
@@ -6702,7 +6711,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>503</v>
       </c>
@@ -6725,7 +6734,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>510</v>
       </c>
@@ -6748,7 +6757,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>516</v>
       </c>
@@ -6771,7 +6780,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="60" customHeight="1">
       <c r="A6" t="s">
         <v>523</v>
       </c>
@@ -6794,7 +6803,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" t="s">
         <v>529</v>
       </c>
@@ -6817,7 +6826,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="60" customHeight="1">
       <c r="A8" t="s">
         <v>535</v>
       </c>
@@ -6840,7 +6849,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="60" customHeight="1">
       <c r="A9" t="s">
         <v>542</v>
       </c>
@@ -6863,7 +6872,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1">
       <c r="A10" t="s">
         <v>549</v>
       </c>
@@ -6886,7 +6895,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1">
       <c r="A11" t="s">
         <v>556</v>
       </c>
@@ -6909,7 +6918,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1">
       <c r="A12" t="s">
         <v>563</v>
       </c>
@@ -6932,7 +6941,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1">
       <c r="A13" t="s">
         <v>570</v>
       </c>
@@ -6955,7 +6964,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1">
       <c r="A14" t="s">
         <v>577</v>
       </c>
@@ -6978,7 +6987,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1">
       <c r="A15" t="s">
         <v>584</v>
       </c>
@@ -7001,7 +7010,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="45" customHeight="1">
       <c r="A16" t="s">
         <v>590</v>
       </c>
@@ -7024,7 +7033,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1">
       <c r="A17" t="s">
         <v>597</v>
       </c>
@@ -7047,7 +7056,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="18" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="45" customHeight="1">
       <c r="A18" t="s">
         <v>604</v>
       </c>
@@ -7070,7 +7079,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1">
       <c r="A19" t="s">
         <v>611</v>
       </c>
@@ -7093,7 +7102,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1">
       <c r="A20" t="s">
         <v>617</v>
       </c>
@@ -7116,7 +7125,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1">
       <c r="A21" t="s">
         <v>622</v>
       </c>
@@ -7139,7 +7148,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="22" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="45" customHeight="1">
       <c r="A22" t="s">
         <v>629</v>
       </c>
@@ -7162,7 +7171,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" customHeight="1">
       <c r="A23" t="s">
         <v>636</v>
       </c>
@@ -7185,7 +7194,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" customHeight="1">
       <c r="A24" t="s">
         <v>643</v>
       </c>
@@ -7208,7 +7217,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" customHeight="1">
       <c r="A25" t="s">
         <v>650</v>
       </c>
@@ -7231,7 +7240,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" customHeight="1">
       <c r="A26" t="s">
         <v>657</v>
       </c>
@@ -7254,7 +7263,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" customHeight="1">
       <c r="A27" t="s">
         <v>664</v>
       </c>
@@ -7277,7 +7286,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="60" customHeight="1">
       <c r="A28" t="s">
         <v>670</v>
       </c>
@@ -7300,7 +7309,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="60" customHeight="1">
       <c r="A29" t="s">
         <v>677</v>
       </c>
@@ -7323,7 +7332,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="60" customHeight="1">
       <c r="A30" t="s">
         <v>684</v>
       </c>
@@ -7346,7 +7355,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60" customHeight="1">
       <c r="A31" t="s">
         <v>691</v>
       </c>
@@ -7369,7 +7378,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="32" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60" customHeight="1">
       <c r="A32" t="s">
         <v>698</v>
       </c>
@@ -7392,7 +7401,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="60" customHeight="1">
       <c r="A33" t="s">
         <v>705</v>
       </c>
@@ -7415,7 +7424,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="60" customHeight="1">
       <c r="A34" t="s">
         <v>712</v>
       </c>
@@ -7438,7 +7447,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="35" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="60" customHeight="1">
       <c r="A35" t="s">
         <v>716</v>
       </c>
@@ -7461,7 +7470,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="60" customHeight="1">
       <c r="A36" t="s">
         <v>723</v>
       </c>
@@ -7484,7 +7493,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="60" customHeight="1">
       <c r="A37" t="s">
         <v>730</v>
       </c>
@@ -7507,7 +7516,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="38" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="60" customHeight="1">
       <c r="A38" t="s">
         <v>737</v>
       </c>
@@ -7530,7 +7539,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="39" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="60" customHeight="1">
       <c r="A39" t="s">
         <v>743</v>
       </c>
@@ -7553,7 +7562,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="60" customHeight="1">
       <c r="A40" t="s">
         <v>750</v>
       </c>
@@ -7576,7 +7585,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="41" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="60" customHeight="1">
       <c r="A41" t="s">
         <v>757</v>
       </c>
@@ -7608,15 +7617,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G54"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" customWidth="1"/>
     <col min="4" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -7639,7 +7648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1">
       <c r="A2" t="s">
         <v>763</v>
       </c>
@@ -7662,7 +7671,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>770</v>
       </c>
@@ -7685,7 +7694,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>777</v>
       </c>
@@ -7708,7 +7717,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>784</v>
       </c>
@@ -7731,7 +7740,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="60" customHeight="1">
       <c r="A6" t="s">
         <v>791</v>
       </c>
@@ -7754,7 +7763,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" t="s">
         <v>798</v>
       </c>
@@ -7777,7 +7786,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="45" customHeight="1">
       <c r="A8" t="s">
         <v>805</v>
       </c>
@@ -7800,7 +7809,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="60" customHeight="1">
       <c r="A9" t="s">
         <v>812</v>
       </c>
@@ -7823,7 +7832,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="45" customHeight="1">
       <c r="A10" t="s">
         <v>819</v>
       </c>
@@ -7846,7 +7855,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1">
       <c r="A11" t="s">
         <v>826</v>
       </c>
@@ -7869,7 +7878,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1">
       <c r="A12" t="s">
         <v>833</v>
       </c>
@@ -7892,7 +7901,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="45" customHeight="1">
       <c r="A13" t="s">
         <v>840</v>
       </c>
@@ -7915,7 +7924,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1">
       <c r="A14" t="s">
         <v>847</v>
       </c>
@@ -7938,7 +7947,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1">
       <c r="A15" t="s">
         <v>854</v>
       </c>
@@ -7961,7 +7970,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1">
       <c r="A16" t="s">
         <v>861</v>
       </c>
@@ -7984,7 +7993,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1">
       <c r="A17" t="s">
         <v>868</v>
       </c>
@@ -8007,7 +8016,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1">
       <c r="A18" t="s">
         <v>875</v>
       </c>
@@ -8030,7 +8039,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1">
       <c r="A19" t="s">
         <v>882</v>
       </c>
@@ -8053,7 +8062,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1">
       <c r="A20" t="s">
         <v>889</v>
       </c>
@@ -8076,7 +8085,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1">
       <c r="A21" t="s">
         <v>896</v>
       </c>
@@ -8099,7 +8108,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60" customHeight="1">
       <c r="A22" t="s">
         <v>903</v>
       </c>
@@ -8122,7 +8131,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" customHeight="1">
       <c r="A23" t="s">
         <v>910</v>
       </c>
@@ -8145,7 +8154,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" customHeight="1">
       <c r="A24" t="s">
         <v>917</v>
       </c>
@@ -8168,7 +8177,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" customHeight="1">
       <c r="A25" t="s">
         <v>924</v>
       </c>
@@ -8191,7 +8200,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" customHeight="1">
       <c r="A26" t="s">
         <v>931</v>
       </c>
@@ -8214,7 +8223,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" customHeight="1">
       <c r="A27" t="s">
         <v>938</v>
       </c>
@@ -8237,7 +8246,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="60" customHeight="1">
       <c r="A28" t="s">
         <v>945</v>
       </c>
@@ -8260,7 +8269,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="29" ht="47.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="47.25" customHeight="1">
       <c r="A29" t="s">
         <v>952</v>
       </c>
@@ -8283,7 +8292,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="60" customHeight="1">
       <c r="A30" t="s">
         <v>959</v>
       </c>
@@ -8306,7 +8315,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60" customHeight="1">
       <c r="A31" t="s">
         <v>966</v>
       </c>
@@ -8329,7 +8338,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="32" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60" customHeight="1">
       <c r="A32" t="s">
         <v>973</v>
       </c>
@@ -8352,7 +8361,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="60" customHeight="1">
       <c r="A33" t="s">
         <v>980</v>
       </c>
@@ -8375,7 +8384,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="60" customHeight="1">
       <c r="A34" t="s">
         <v>987</v>
       </c>
@@ -8398,7 +8407,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="35" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="45" customHeight="1">
       <c r="A35" t="s">
         <v>994</v>
       </c>
@@ -8421,7 +8430,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="60" customHeight="1">
       <c r="A36" t="s">
         <v>1001</v>
       </c>
@@ -8444,7 +8453,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="37" ht="62.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="62.25" customHeight="1">
       <c r="A37" t="s">
         <v>1008</v>
       </c>
@@ -8467,7 +8476,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="38" ht="47.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="47.25" customHeight="1">
       <c r="A38" t="s">
         <v>1015</v>
       </c>
@@ -8490,7 +8499,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="39" ht="50.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="50.25" customHeight="1">
       <c r="A39" t="s">
         <v>1022</v>
       </c>
@@ -8513,7 +8522,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="60" customHeight="1">
       <c r="A40" t="s">
         <v>1029</v>
       </c>
@@ -8536,7 +8545,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="41" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="60" customHeight="1">
       <c r="A41" t="s">
         <v>1036</v>
       </c>
@@ -8559,7 +8568,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="42" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="60" customHeight="1">
       <c r="A42" t="s">
         <v>1041</v>
       </c>
@@ -8582,7 +8591,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="43" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="60" customHeight="1">
       <c r="A43" t="s">
         <v>1048</v>
       </c>
@@ -8605,7 +8614,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="44" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="45" customHeight="1">
       <c r="A44" t="s">
         <v>1055</v>
       </c>
@@ -8628,7 +8637,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="45" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="60" customHeight="1">
       <c r="A45" t="s">
         <v>1062</v>
       </c>
@@ -8651,7 +8660,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="60" customHeight="1">
       <c r="A46" t="s">
         <v>1069</v>
       </c>
@@ -8674,7 +8683,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="47" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="60" customHeight="1">
       <c r="A47" t="s">
         <v>1076</v>
       </c>
@@ -8697,7 +8706,7 @@
         <v>1082</v>
       </c>
     </row>
-    <row r="48" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="60" customHeight="1">
       <c r="A48" t="s">
         <v>1083</v>
       </c>
@@ -8720,7 +8729,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="49" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="60" customHeight="1">
       <c r="A49" t="s">
         <v>1090</v>
       </c>
@@ -8743,7 +8752,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="50" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="45" customHeight="1">
       <c r="A50" t="s">
         <v>1097</v>
       </c>
@@ -8766,7 +8775,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="51" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="60" customHeight="1">
       <c r="A51" t="s">
         <v>1104</v>
       </c>
@@ -8789,7 +8798,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="52" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="60" customHeight="1">
       <c r="A52" t="s">
         <v>1111</v>
       </c>
@@ -8812,7 +8821,7 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="53" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="60" customHeight="1">
       <c r="A53" t="s">
         <v>1118</v>
       </c>
@@ -8835,7 +8844,7 @@
         <v>1124</v>
       </c>
     </row>
-    <row r="54" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="60" customHeight="1">
       <c r="A54" t="s">
         <v>1125</v>
       </c>
@@ -8867,15 +8876,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" customWidth="1"/>
     <col min="4" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -8898,7 +8907,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1">
       <c r="A2" t="s">
         <v>1132</v>
       </c>
@@ -8921,7 +8930,7 @@
         <v>1138</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>1139</v>
       </c>
@@ -8944,7 +8953,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>1146</v>
       </c>
@@ -8967,7 +8976,7 @@
         <v>1152</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>1153</v>
       </c>
@@ -8990,7 +8999,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="60" customHeight="1">
       <c r="A6" t="s">
         <v>1159</v>
       </c>
@@ -9013,7 +9022,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" t="s">
         <v>1166</v>
       </c>
@@ -9036,7 +9045,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="60" customHeight="1">
       <c r="A8" t="s">
         <v>1173</v>
       </c>
@@ -9059,7 +9068,7 @@
         <v>1179</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="60" customHeight="1">
       <c r="A9" t="s">
         <v>1180</v>
       </c>
@@ -9082,7 +9091,7 @@
         <v>1186</v>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1">
       <c r="A10" t="s">
         <v>1187</v>
       </c>
@@ -9105,7 +9114,7 @@
         <v>1193</v>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1">
       <c r="A11" t="s">
         <v>1194</v>
       </c>
@@ -9128,7 +9137,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1">
       <c r="A12" t="s">
         <v>1201</v>
       </c>
@@ -9151,7 +9160,7 @@
         <v>1206</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1">
       <c r="A13" t="s">
         <v>1207</v>
       </c>
@@ -9174,7 +9183,7 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1">
       <c r="A14" t="s">
         <v>1214</v>
       </c>
@@ -9197,7 +9206,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1">
       <c r="A15" t="s">
         <v>1221</v>
       </c>
@@ -9220,7 +9229,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1">
       <c r="A16" t="s">
         <v>1228</v>
       </c>
@@ -9243,7 +9252,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1">
       <c r="A17" t="s">
         <v>1235</v>
       </c>
@@ -9266,7 +9275,7 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1">
       <c r="A18" t="s">
         <v>1242</v>
       </c>
@@ -9289,7 +9298,7 @@
         <v>1248</v>
       </c>
     </row>
-    <row r="19" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="45" customHeight="1">
       <c r="A19" t="s">
         <v>1249</v>
       </c>
@@ -9312,7 +9321,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1">
       <c r="A20" t="s">
         <v>1256</v>
       </c>
@@ -9335,7 +9344,7 @@
         <v>1262</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1">
       <c r="A21" t="s">
         <v>1263</v>
       </c>
@@ -9358,7 +9367,7 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60" customHeight="1">
       <c r="A22" t="s">
         <v>1270</v>
       </c>
@@ -9381,7 +9390,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" customHeight="1">
       <c r="A23" t="s">
         <v>1277</v>
       </c>
@@ -9404,7 +9413,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" customHeight="1">
       <c r="A24" t="s">
         <v>1284</v>
       </c>
@@ -9427,7 +9436,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" customHeight="1">
       <c r="A25" t="s">
         <v>1291</v>
       </c>
@@ -9450,7 +9459,7 @@
         <v>1297</v>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" customHeight="1">
       <c r="A26" t="s">
         <v>1298</v>
       </c>
@@ -9473,7 +9482,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" customHeight="1">
       <c r="A27" t="s">
         <v>1305</v>
       </c>
@@ -9505,15 +9514,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
     <col min="4" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -9536,7 +9545,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="45" customHeight="1">
       <c r="A2" t="s">
         <v>1312</v>
       </c>
@@ -9559,7 +9568,7 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>1319</v>
       </c>
@@ -9582,7 +9591,7 @@
         <v>1325</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>1326</v>
       </c>
@@ -9605,7 +9614,7 @@
         <v>1332</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>1333</v>
       </c>
@@ -9628,7 +9637,7 @@
         <v>1339</v>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="60" customHeight="1">
       <c r="A6" t="s">
         <v>1340</v>
       </c>
@@ -9660,7 +9669,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -9668,7 +9677,7 @@
     <col min="7" max="7" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -9691,7 +9700,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1">
       <c r="A2" t="s">
         <v>1347</v>
       </c>
@@ -9714,7 +9723,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1">
       <c r="A3" t="s">
         <v>1354</v>
       </c>
@@ -9737,7 +9746,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1">
       <c r="A4" t="s">
         <v>1361</v>
       </c>
@@ -9760,7 +9769,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="60" customHeight="1">
       <c r="A5" t="s">
         <v>1368</v>
       </c>
@@ -9783,7 +9792,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="60" customHeight="1">
       <c r="A6" t="s">
         <v>1375</v>
       </c>
@@ -9806,7 +9815,7 @@
         <v>1381</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" customHeight="1">
       <c r="A7" t="s">
         <v>1382</v>
       </c>
@@ -9829,7 +9838,7 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="60" customHeight="1">
       <c r="A8" t="s">
         <v>1389</v>
       </c>
@@ -9852,7 +9861,7 @@
         <v>1395</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="60" customHeight="1">
       <c r="A9" t="s">
         <v>1396</v>
       </c>
@@ -9875,7 +9884,7 @@
         <v>1402</v>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1">
       <c r="A10" t="s">
         <v>1403</v>
       </c>
@@ -9898,7 +9907,7 @@
         <v>1409</v>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="45" customHeight="1">
       <c r="A11" t="s">
         <v>1410</v>
       </c>
@@ -9921,7 +9930,7 @@
         <v>1416</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1">
       <c r="A12" t="s">
         <v>1417</v>
       </c>
@@ -9944,7 +9953,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1">
       <c r="A13" t="s">
         <v>1424</v>
       </c>
@@ -9967,7 +9976,7 @@
         <v>1430</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1">
       <c r="A14" t="s">
         <v>1431</v>
       </c>
@@ -9990,7 +9999,7 @@
         <v>1437</v>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1">
       <c r="A15" t="s">
         <v>1438</v>
       </c>
@@ -10013,7 +10022,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1">
       <c r="A16" t="s">
         <v>1445</v>
       </c>
@@ -10036,7 +10045,7 @@
         <v>1451</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1">
       <c r="A17" t="s">
         <v>1452</v>
       </c>
@@ -10059,7 +10068,7 @@
         <v>1458</v>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1">
       <c r="A18" t="s">
         <v>1459</v>
       </c>
@@ -10082,7 +10091,7 @@
         <v>1465</v>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1">
       <c r="A19" t="s">
         <v>1466</v>
       </c>
@@ -10105,7 +10114,7 @@
         <v>1472</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1">
       <c r="A20" t="s">
         <v>1473</v>
       </c>
@@ -10128,7 +10137,7 @@
         <v>1479</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1">
       <c r="A21" t="s">
         <v>1480</v>
       </c>
@@ -10159,8 +10168,8 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>